<commit_message>
docs(staging): remove published super-admin credentials from runbook and test manual
The staging super-admin email and password were published in the public
repository since 497af377 (2026-05-21). The account password was reset on
2026-09-26 (staging only) and the new secret is held outside the repository.

- STAGING_WORKFLOW.md: replace the credentials with the access procedure.
- generate_test_artifacts.py: replace the credential strings.
- Regenerate staging_validation_test_manual.pdf and
  staging_validation_test_cases.xlsx from the updated generator.

History is not rewritten; the old password is refused by staging.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/release/testing/staging_validation_test_cases.xlsx
+++ b/docs/release/testing/staging_validation_test_cases.xlsx
@@ -928,7 +928,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>admin@promoshake.net / Admin1234!</t>
+          <t>Super admin credentials from the staging owner (never versioned)</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-09-26</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>admin@promoshake.net  /  Admin1234!</t>
+          <t>super admin credentials: ask the staging owner (never versioned)</t>
         </is>
       </c>
     </row>

</xml_diff>